<commit_message>
Add wiki_kb system, user project RAG, LibreOffice for .doc support, per-role session generation
- wiki_kb: full Karpathy RAG pipeline (ingest, corpus analysis, compile, index, ask)
- Library: integrated wiki query chatbot + user project upload/rebuild workflow
- Dashboard: PM can trigger per-engineer session generation (process/mechanical independently)
- server.js: user project CRUD, file management, rebuild, role-filtered suggest-sessions
- Dockerfile/nixpacks: add libreoffice-writer for .doc → .docx conversion on Railway
- .gitignore: exclude node_modules, user_projects, wiki_kb/db, parsed caches

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/work_agents/Aria - Process Engineer/deliverables/1-CAL-XXXX.xlsx
+++ b/work_agents/Aria - Process Engineer/deliverables/1-CAL-XXXX.xlsx
@@ -813,7 +813,7 @@
         </is>
       </c>
       <c r="C13" s="13" t="n">
-        <v>4</v>
+        <v>2.5</v>
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="C14" s="13" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="D14" s="12" t="inlineStr">
         <is>
@@ -866,7 +866,7 @@
       </c>
       <c r="C15" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
@@ -894,7 +894,7 @@
       </c>
       <c r="C16" s="17" t="inlineStr">
         <is>
-          <t>Monoethylene Glycol (MEG) requires corrosion inhibition, especially at elevated temperatures and in the presence of oxygen, to prevent degradation and the formation of corrosive organic acids. It is also hygroscopic and can absorb water from the atmosphere.</t>
+          <t>MEG is hygroscopic and can degrade to corrosive organic acids (e.g., glycolic acid) over time, especially in the presence of oxygen and high temperatures. Inhibition is often required for long-term use in carbon steel systems. Ensure proper material selection and monitoring.</t>
         </is>
       </c>
       <c r="D16" s="16" t="inlineStr">
@@ -1652,7 +1652,7 @@
     <row r="50">
       <c r="A50" s="27" t="inlineStr">
         <is>
-          <t>Generated by Process Engineer Agent (Aria)  |  2026-04-02T18:32:46  |  A Star Chemical</t>
+          <t>Generated by Process Engineer Agent (Aria)  |  2026-04-02T23:09:13  |  A Star Chemical</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: electrical engines + reusable calc xlsx template
- engines/: load_density (DPS density, cable/VD), load_itemized (IEC),
  transformer (short-circuit + loading), panelboard, cable_vd, refstd, db
  (SQLite + change propagation), ref_tables (dps/iec/cable_vd/panel_lv),
  fixtures, golden tests (159 passing)
- Nova electrical agent: runs load/transformer/panelboard, --change-room propagation
- export_xlsx: reusable 4-sheet electrical calc workbook (Cover/Load-Calc/
  Summary/Ref-Tables) with live formulas referencing Ref-Tables (877 kVA)
- server.js/Dashboard: electrical panels, cable/VD columns, propagation,
  missing-input hints; commercial_building catalog + full-discipline PM

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/work_agents/Aria - Process Engineer/deliverables/1-CAL-XXXX.xlsx
+++ b/work_agents/Aria - Process Engineer/deliverables/1-CAL-XXXX.xlsx
@@ -649,7 +649,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Sarnia, Ontario, Canada</t>
+          <t>Sarnia, Canada</t>
         </is>
       </c>
       <c r="C5" s="7" t="n"/>
@@ -665,7 +665,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="C6" s="7" t="n"/>
@@ -813,7 +813,7 @@
         </is>
       </c>
       <c r="C13" s="13" t="n">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="C14" s="13" t="n">
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
       <c r="D14" s="12" t="inlineStr">
         <is>
@@ -866,7 +866,7 @@
       </c>
       <c r="C15" s="13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
@@ -894,7 +894,7 @@
       </c>
       <c r="C16" s="17" t="inlineStr">
         <is>
-          <t>MEG is hygroscopic and can degrade to corrosive organic acids (e.g., glycolic acid) over time, especially in the presence of oxygen and high temperatures. Inhibition is often required for long-term use in carbon steel systems. Ensure proper material selection and monitoring.</t>
+          <t>MEG is hygroscopic and can degrade to corrosive organic acids (e.g., glycolic acid) at elevated temperatures or in the presence of oxygen. Proper inhibition and material selection are crucial to prevent corrosion. Viscosity and vapor pressure are engineering estimates for 95% MEG at 65 °C.</t>
         </is>
       </c>
       <c r="D16" s="16" t="inlineStr">
@@ -1251,7 +1251,7 @@
         </is>
       </c>
       <c r="C31" s="13" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="D31" s="12" t="inlineStr">
         <is>
@@ -1261,7 +1261,7 @@
       <c r="E31" s="14" t="inlineStr"/>
       <c r="F31" s="14" t="inlineStr">
         <is>
-          <t>Source: 5-LST-0003</t>
+          <t>Source: 5-LST-0003-2</t>
         </is>
       </c>
     </row>
@@ -1652,7 +1652,7 @@
     <row r="50">
       <c r="A50" s="27" t="inlineStr">
         <is>
-          <t>Generated by Process Engineer Agent (Aria)  |  2026-04-02T23:09:13  |  A Star Chemical</t>
+          <t>Generated by Process Engineer Agent (Aria)  |  2026-04-28T04:08:00  |  A Star Chemical</t>
         </is>
       </c>
     </row>

</xml_diff>